<commit_message>
13 data points collected so far
</commit_message>
<xml_diff>
--- a/Dear_Data_Project/sibling_data.xlsx
+++ b/Dear_Data_Project/sibling_data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/4072360cc263ec0b/Processing/DearDataProject/Dear Data Project/Dear_Data_Project/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="6" documentId="8_{F06C03BE-BA34-4718-934D-620FB05A1E63}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EE2B1E3A-79EB-4584-BADA-2A18F06E03F0}"/>
+  <xr:revisionPtr revIDLastSave="8" documentId="8_{F06C03BE-BA34-4718-934D-620FB05A1E63}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{72C818CE-7318-412D-9ECF-270948028368}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="48">
   <si>
     <t>ID</t>
   </si>
@@ -40,9 +40,6 @@
     <t>Duration (mins)</t>
   </si>
   <si>
-    <t>Argued / Conflict</t>
-  </si>
-  <si>
     <t>Sister</t>
   </si>
   <si>
@@ -110,6 +107,63 @@
   </si>
   <si>
     <t>Shared Activity / help</t>
+  </si>
+  <si>
+    <t>Time of day</t>
+  </si>
+  <si>
+    <t>Argued / Conflict/food</t>
+  </si>
+  <si>
+    <t>Night</t>
+  </si>
+  <si>
+    <t>Evening</t>
+  </si>
+  <si>
+    <t>Afternoon</t>
+  </si>
+  <si>
+    <t>Morning</t>
+  </si>
+  <si>
+    <t>Watched BetaSquad together</t>
+  </si>
+  <si>
+    <t>shared activity/screen</t>
+  </si>
+  <si>
+    <t>Dining room</t>
+  </si>
+  <si>
+    <t>Did homework together</t>
+  </si>
+  <si>
+    <t>shared activity/help</t>
+  </si>
+  <si>
+    <t>Ate dinner together</t>
+  </si>
+  <si>
+    <t>Shared Activity/food</t>
+  </si>
+  <si>
+    <t>Complained about food at dinnertime</t>
+  </si>
+  <si>
+    <t>vent/gossip/food</t>
+  </si>
+  <si>
+    <t>Played roblox together</t>
+  </si>
+  <si>
+    <t>Online/Fun</t>
+  </si>
+  <si>
+    <t>Tucked sister into bed and read a book</t>
+  </si>
+  <si>
+    <t>Bonding/Help</t>
   </si>
 </sst>
 </file>
@@ -149,7 +203,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -172,17 +226,31 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFD9D9D9"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFD9D9D9"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="14" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -198,6 +266,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -485,7 +557,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G8"/>
+  <dimension ref="A1:H14"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -497,7 +569,7 @@
     <col min="7" max="7" width="22" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -517,10 +589,13 @@
         <v>5</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+        <v>18</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A2" s="2">
         <v>1</v>
       </c>
@@ -528,22 +603,25 @@
         <v>46303</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D2" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="E2" s="2" t="s">
         <v>6</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>7</v>
       </c>
       <c r="F2" s="2">
         <v>10</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+        <v>12</v>
+      </c>
+      <c r="H2" s="4" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3" s="2">
         <v>2</v>
       </c>
@@ -551,22 +629,25 @@
         <v>46304</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D3" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E3" s="2" t="s">
         <v>9</v>
-      </c>
-      <c r="E3" s="2" t="s">
-        <v>10</v>
       </c>
       <c r="F3" s="2">
         <v>15</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+        <v>10</v>
+      </c>
+      <c r="H3" s="4" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A4" s="2">
         <v>3</v>
       </c>
@@ -574,22 +655,25 @@
         <v>46304</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F4" s="2">
         <v>25</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+        <v>22</v>
+      </c>
+      <c r="H4" s="4" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A5" s="2">
         <v>4</v>
       </c>
@@ -597,22 +681,25 @@
         <v>46305</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D5" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E5" s="2" t="s">
         <v>14</v>
-      </c>
-      <c r="E5" s="2" t="s">
-        <v>15</v>
       </c>
       <c r="F5" s="2">
         <v>100</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+        <v>12</v>
+      </c>
+      <c r="H5" s="5" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A6" s="2">
         <v>5</v>
       </c>
@@ -620,22 +707,25 @@
         <v>46305</v>
       </c>
       <c r="C6" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="D6" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="D6" s="2" t="s">
-        <v>17</v>
-      </c>
       <c r="E6" s="2" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F6" s="2">
         <v>3</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+        <v>7</v>
+      </c>
+      <c r="H6" s="5" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A7" s="2">
         <v>6</v>
       </c>
@@ -643,22 +733,25 @@
         <v>46306</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="F7" s="2">
         <v>180</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+        <v>25</v>
+      </c>
+      <c r="H7" s="5" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A8" s="2">
         <v>7</v>
       </c>
@@ -666,19 +759,178 @@
         <v>46306</v>
       </c>
       <c r="C8" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="D8" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="D8" s="2" t="s">
-        <v>29</v>
-      </c>
       <c r="E8" s="2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="F8" s="2">
         <v>40</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>18</v>
+        <v>17</v>
+      </c>
+      <c r="H8" s="5" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A9" s="4">
+        <v>8</v>
+      </c>
+      <c r="B9" s="6">
+        <v>46307</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="D9" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="E9" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="F9" s="4">
+        <v>30</v>
+      </c>
+      <c r="G9" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="H9" s="5" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A10" s="4">
+        <v>9</v>
+      </c>
+      <c r="B10" s="6">
+        <v>46307</v>
+      </c>
+      <c r="C10" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="D10" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="E10" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="F10" s="4">
+        <v>120</v>
+      </c>
+      <c r="G10" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="H10" s="5" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A11" s="4">
+        <v>10</v>
+      </c>
+      <c r="B11" s="6">
+        <v>46308</v>
+      </c>
+      <c r="C11" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="D11" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="E11" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="F11" s="4">
+        <v>40</v>
+      </c>
+      <c r="G11" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="H11" s="5" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A12" s="4">
+        <v>11</v>
+      </c>
+      <c r="B12" s="6">
+        <v>46308</v>
+      </c>
+      <c r="C12" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="D12" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="E12" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="F12" s="4">
+        <v>15</v>
+      </c>
+      <c r="G12" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="H12" s="5" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A13" s="4">
+        <v>12</v>
+      </c>
+      <c r="B13" s="6">
+        <v>46308</v>
+      </c>
+      <c r="C13" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="D13" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="E13" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="F13" s="4">
+        <v>75</v>
+      </c>
+      <c r="G13" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="H13" s="5" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A14" s="4">
+        <v>13</v>
+      </c>
+      <c r="B14" s="6">
+        <v>46308</v>
+      </c>
+      <c r="C14" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="D14" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="E14" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="F14" s="4">
+        <v>20</v>
+      </c>
+      <c r="G14" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="H14" s="5" t="s">
+        <v>31</v>
       </c>
     </row>
   </sheetData>
@@ -687,6 +939,21 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100E802F14A90D1B345818A6FFB06D8A03D" ma:contentTypeVersion="4" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ea7226ff09ef22af6f5ba21dc65cff36">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="75eb23ce-bee3-4614-ac9d-e7493ba98713" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="807d9844cc6c643302a5e086dcc98a76" ns3:_="">
     <xsd:import namespace="75eb23ce-bee3-4614-ac9d-e7493ba98713"/>
@@ -830,22 +1097,31 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B15FDCE2-C38D-4DD1-B711-A8CB81A27211}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="75eb23ce-bee3-4614-ac9d-e7493ba98713"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{33023472-F23D-4624-BC7A-4AE1438DE3EC}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{997A7A74-A1F7-48AE-82CD-9856C622E446}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -861,28 +1137,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{33023472-F23D-4624-BC7A-4AE1438DE3EC}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B15FDCE2-C38D-4DD1-B711-A8CB81A27211}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="75eb23ce-bee3-4614-ac9d-e7493ba98713"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
size + background modified
</commit_message>
<xml_diff>
--- a/Dear_Data_Project/sibling_data.xlsx
+++ b/Dear_Data_Project/sibling_data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/4072360cc263ec0b/Processing/DearDataProject/Dear Data Project/Dear_Data_Project/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="35" documentId="8_{F06C03BE-BA34-4718-934D-620FB05A1E63}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F3B6AF72-DE54-4DC2-A6FD-F89621DA1B54}"/>
+  <xr:revisionPtr revIDLastSave="66" documentId="8_{F06C03BE-BA34-4718-934D-620FB05A1E63}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DD9EB37A-5713-4915-B935-BC7A8A0B24F7}"/>
   <bookViews>
-    <workbookView minimized="1" xWindow="3660" yWindow="2316" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sibling Interactions" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="109" uniqueCount="70">
   <si>
     <t>ID</t>
   </si>
@@ -195,6 +195,54 @@
   </si>
   <si>
     <t>both</t>
+  </si>
+  <si>
+    <t>Positivity Scale(1-10)</t>
+  </si>
+  <si>
+    <t>My mood</t>
+  </si>
+  <si>
+    <t>Her mood</t>
+  </si>
+  <si>
+    <t>Angry</t>
+  </si>
+  <si>
+    <t>Happy</t>
+  </si>
+  <si>
+    <t>calm</t>
+  </si>
+  <si>
+    <t>excited</t>
+  </si>
+  <si>
+    <t>exhausted</t>
+  </si>
+  <si>
+    <t>energised</t>
+  </si>
+  <si>
+    <t>happy</t>
+  </si>
+  <si>
+    <t>stressed</t>
+  </si>
+  <si>
+    <t>upset</t>
+  </si>
+  <si>
+    <t>enthusiastic</t>
+  </si>
+  <si>
+    <t>relaxed</t>
+  </si>
+  <si>
+    <t>angry</t>
+  </si>
+  <si>
+    <t>entertained</t>
   </si>
 </sst>
 </file>
@@ -234,7 +282,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -268,11 +316,20 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFD9D9D9"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -282,7 +339,8 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -589,7 +647,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H51"/>
+  <dimension ref="A1:K51"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -601,7 +659,7 @@
     <col min="7" max="7" width="22" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -626,8 +684,17 @@
       <c r="H1" s="1" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I1" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A2" s="2">
         <v>1</v>
       </c>
@@ -652,8 +719,17 @@
       <c r="H2" s="4" t="s">
         <v>32</v>
       </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I2">
+        <v>2</v>
+      </c>
+      <c r="J2" s="7" t="s">
+        <v>57</v>
+      </c>
+      <c r="K2" s="7" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A3" s="2">
         <v>2</v>
       </c>
@@ -678,8 +754,17 @@
       <c r="H3" s="4" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I3">
+        <v>10</v>
+      </c>
+      <c r="J3" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="K3" s="7" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A4" s="2">
         <v>3</v>
       </c>
@@ -704,8 +789,14 @@
       <c r="H4" s="4" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I4">
+        <v>9</v>
+      </c>
+      <c r="J4" s="7" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A5" s="2">
         <v>4</v>
       </c>
@@ -730,8 +821,14 @@
       <c r="H5" s="5" t="s">
         <v>34</v>
       </c>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I5">
+        <v>10</v>
+      </c>
+      <c r="J5" s="8" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A6" s="2">
         <v>5</v>
       </c>
@@ -756,8 +853,14 @@
       <c r="H6" s="5" t="s">
         <v>34</v>
       </c>
-    </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I6">
+        <v>1</v>
+      </c>
+      <c r="J6" s="8" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A7" s="2">
         <v>6</v>
       </c>
@@ -782,8 +885,14 @@
       <c r="H7" s="5" t="s">
         <v>35</v>
       </c>
-    </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I7">
+        <v>10</v>
+      </c>
+      <c r="J7" s="8" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A8" s="2">
         <v>7</v>
       </c>
@@ -808,8 +917,14 @@
       <c r="H8" s="5" t="s">
         <v>32</v>
       </c>
-    </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I8">
+        <v>9</v>
+      </c>
+      <c r="J8" s="8" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A9" s="4">
         <v>8</v>
       </c>
@@ -834,8 +949,14 @@
       <c r="H9" s="5" t="s">
         <v>32</v>
       </c>
-    </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I9">
+        <v>10</v>
+      </c>
+      <c r="J9" s="8" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A10" s="4">
         <v>9</v>
       </c>
@@ -860,8 +981,14 @@
       <c r="H10" s="5" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I10">
+        <v>7</v>
+      </c>
+      <c r="J10" s="8" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A11" s="4">
         <v>10</v>
       </c>
@@ -886,8 +1013,14 @@
       <c r="H11" s="5" t="s">
         <v>32</v>
       </c>
-    </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I11">
+        <v>9</v>
+      </c>
+      <c r="J11" s="8" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A12" s="4">
         <v>11</v>
       </c>
@@ -912,8 +1045,14 @@
       <c r="H12" s="5" t="s">
         <v>32</v>
       </c>
-    </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I12">
+        <v>3</v>
+      </c>
+      <c r="J12" s="8" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A13" s="4">
         <v>12</v>
       </c>
@@ -938,8 +1077,14 @@
       <c r="H13" s="5" t="s">
         <v>32</v>
       </c>
-    </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I13">
+        <v>10</v>
+      </c>
+      <c r="J13" s="8" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A14" s="4">
         <v>13</v>
       </c>
@@ -964,8 +1109,14 @@
       <c r="H14" s="5" t="s">
         <v>32</v>
       </c>
-    </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I14">
+        <v>10</v>
+      </c>
+      <c r="J14" s="8" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A15">
         <f>SUM(A14,1)</f>
         <v>14</v>
@@ -973,26 +1124,32 @@
       <c r="B15" s="6">
         <v>46309</v>
       </c>
-      <c r="C15" s="7" t="s">
+      <c r="C15" s="4" t="s">
         <v>49</v>
       </c>
-      <c r="D15" s="7" t="s">
+      <c r="D15" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="E15" s="7" t="s">
+      <c r="E15" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="F15" s="7">
+      <c r="F15" s="4">
         <v>7</v>
       </c>
-      <c r="G15" s="7" t="s">
+      <c r="G15" s="4" t="s">
         <v>50</v>
       </c>
       <c r="H15" s="5" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I15">
+        <v>0</v>
+      </c>
+      <c r="J15" s="8" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A16">
         <f t="shared" ref="A16:A51" si="0">SUM(A15,1)</f>
         <v>15</v>
@@ -1000,26 +1157,32 @@
       <c r="B16" s="6">
         <v>46309</v>
       </c>
-      <c r="C16" s="7" t="s">
+      <c r="C16" s="4" t="s">
         <v>51</v>
       </c>
-      <c r="D16" s="7" t="s">
+      <c r="D16" s="4" t="s">
         <v>52</v>
       </c>
-      <c r="E16" s="7" t="s">
+      <c r="E16" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="F16" s="7">
+      <c r="F16" s="4">
         <v>35</v>
       </c>
-      <c r="G16" s="7" t="s">
+      <c r="G16" s="4" t="s">
         <v>13</v>
       </c>
       <c r="H16" s="5" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I16">
+        <v>9</v>
+      </c>
+      <c r="J16" s="8" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="17" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A17">
         <f t="shared" si="0"/>
         <v>16</v>
@@ -1027,110 +1190,128 @@
       <c r="B17" s="6">
         <v>46309</v>
       </c>
-      <c r="C17" s="7" t="s">
+      <c r="C17" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="D17" s="7" t="s">
+      <c r="D17" s="4" t="s">
         <v>52</v>
       </c>
-      <c r="E17" s="7" t="s">
+      <c r="E17" s="4" t="s">
         <v>53</v>
       </c>
-      <c r="F17" s="7">
+      <c r="F17" s="4">
         <v>40</v>
       </c>
-      <c r="G17" s="7" t="s">
+      <c r="G17" s="4" t="s">
         <v>13</v>
       </c>
       <c r="H17" s="5" t="s">
         <v>32</v>
       </c>
-    </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I17">
+        <v>9</v>
+      </c>
+      <c r="J17" s="8" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="18" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A18">
         <f t="shared" si="0"/>
         <v>17</v>
       </c>
-    </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="B18" s="6">
+        <v>46310</v>
+      </c>
+    </row>
+    <row r="19" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A19">
         <f t="shared" si="0"/>
         <v>18</v>
       </c>
-    </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="B19" s="6">
+        <v>46310</v>
+      </c>
+    </row>
+    <row r="20" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A20">
         <f t="shared" si="0"/>
         <v>19</v>
       </c>
-    </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="B20" s="6">
+        <v>46310</v>
+      </c>
+    </row>
+    <row r="21" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A21">
         <f t="shared" si="0"/>
         <v>20</v>
       </c>
-    </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="B21" s="6">
+        <v>46310</v>
+      </c>
+    </row>
+    <row r="22" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A22">
         <f t="shared" si="0"/>
         <v>21</v>
       </c>
     </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A23">
         <f t="shared" si="0"/>
         <v>22</v>
       </c>
     </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A24">
         <f t="shared" si="0"/>
         <v>23</v>
       </c>
     </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A25">
         <f t="shared" si="0"/>
         <v>24</v>
       </c>
     </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A26">
         <f t="shared" si="0"/>
         <v>25</v>
       </c>
     </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A27">
         <f t="shared" si="0"/>
         <v>26</v>
       </c>
     </row>
-    <row r="28" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A28">
         <f t="shared" si="0"/>
         <v>27</v>
       </c>
     </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A29">
         <f t="shared" si="0"/>
         <v>28</v>
       </c>
     </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A30">
         <f t="shared" si="0"/>
         <v>29</v>
       </c>
     </row>
-    <row r="31" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A31">
         <f t="shared" si="0"/>
         <v>30</v>
       </c>
     </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A32">
         <f t="shared" si="0"/>
         <v>31</v>
@@ -1262,15 +1443,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100E802F14A90D1B345818A6FFB06D8A03D" ma:contentTypeVersion="4" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ea7226ff09ef22af6f5ba21dc65cff36">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="75eb23ce-bee3-4614-ac9d-e7493ba98713" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="807d9844cc6c643302a5e086dcc98a76" ns3:_="">
     <xsd:import namespace="75eb23ce-bee3-4614-ac9d-e7493ba98713"/>
@@ -1414,6 +1586,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B15FDCE2-C38D-4DD1-B711-A8CB81A27211}">
   <ds:schemaRefs>
@@ -1431,14 +1612,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{33023472-F23D-4624-BC7A-4AE1438DE3EC}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{997A7A74-A1F7-48AE-82CD-9856C622E446}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1454,4 +1627,12 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{33023472-F23D-4624-BC7A-4AE1438DE3EC}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
29 data points and sketch plan
</commit_message>
<xml_diff>
--- a/Dear_Data_Project/sibling_data.xlsx
+++ b/Dear_Data_Project/sibling_data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/4072360cc263ec0b/Processing/DearDataProject/Dear Data Project/Dear_Data_Project/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="66" documentId="8_{F06C03BE-BA34-4718-934D-620FB05A1E63}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DD9EB37A-5713-4915-B935-BC7A8A0B24F7}"/>
+  <xr:revisionPtr revIDLastSave="205" documentId="8_{F06C03BE-BA34-4718-934D-620FB05A1E63}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B25BE202-2DB5-4D1C-B1FC-0CB240600BDF}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="109" uniqueCount="70">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="174" uniqueCount="87">
   <si>
     <t>ID</t>
   </si>
@@ -53,18 +53,12 @@
     <t>Duration (mins)</t>
   </si>
   <si>
-    <t>Argued / Conflict</t>
-  </si>
-  <si>
     <t>Sister</t>
   </si>
   <si>
     <t>Living Room</t>
   </si>
   <si>
-    <t>Laughed / Fun</t>
-  </si>
-  <si>
     <t>Me</t>
   </si>
   <si>
@@ -83,12 +77,6 @@
     <t>Both</t>
   </si>
   <si>
-    <t>Complained about household chores</t>
-  </si>
-  <si>
-    <t>Vent / Gossip</t>
-  </si>
-  <si>
     <t>Bedroom</t>
   </si>
   <si>
@@ -116,9 +104,6 @@
     <t>outdoors(swimming pool)</t>
   </si>
   <si>
-    <t>sport/exercise</t>
-  </si>
-  <si>
     <t>dressed up together</t>
   </si>
   <si>
@@ -128,9 +113,6 @@
     <t>Time of day</t>
   </si>
   <si>
-    <t>Argued / Conflict/food</t>
-  </si>
-  <si>
     <t>Night</t>
   </si>
   <si>
@@ -143,12 +125,6 @@
     <t>Morning</t>
   </si>
   <si>
-    <t>Watched BetaSquad together</t>
-  </si>
-  <si>
-    <t>shared activity/screen</t>
-  </si>
-  <si>
     <t>Dining room</t>
   </si>
   <si>
@@ -161,21 +137,12 @@
     <t>Ate dinner together</t>
   </si>
   <si>
-    <t>Shared Activity/food</t>
-  </si>
-  <si>
     <t>Complained about food at dinnertime</t>
   </si>
   <si>
-    <t>vent/gossip/food</t>
-  </si>
-  <si>
     <t>Played roblox together</t>
   </si>
   <si>
-    <t>Online/Fun</t>
-  </si>
-  <si>
     <t>Tucked sister into bed and read a book</t>
   </si>
   <si>
@@ -191,9 +158,6 @@
     <t>Cooked dinner together</t>
   </si>
   <si>
-    <t>Shared activity/food</t>
-  </si>
-  <si>
     <t>both</t>
   </si>
   <si>
@@ -243,6 +207,93 @@
   </si>
   <si>
     <t>entertained</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Watched a movie together </t>
+  </si>
+  <si>
+    <t>Outdoors/theatre</t>
+  </si>
+  <si>
+    <t>Played arcade games</t>
+  </si>
+  <si>
+    <t>Entertainment</t>
+  </si>
+  <si>
+    <t>Outdoors</t>
+  </si>
+  <si>
+    <t>Watched BetaSquad together while eating</t>
+  </si>
+  <si>
+    <t>Complained about household chores during dinner</t>
+  </si>
+  <si>
+    <t>Food</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Night </t>
+  </si>
+  <si>
+    <t>Vent / Gossip/Food(x3)</t>
+  </si>
+  <si>
+    <t>Shared activity/help</t>
+  </si>
+  <si>
+    <t xml:space="preserve">played football </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Conflict/food</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Fun</t>
+  </si>
+  <si>
+    <t>Sport</t>
+  </si>
+  <si>
+    <t>food</t>
+  </si>
+  <si>
+    <t>gossip/food</t>
+  </si>
+  <si>
+    <t>Online/Entertainment</t>
+  </si>
+  <si>
+    <t>Conflict</t>
+  </si>
+  <si>
+    <t>Fun</t>
+  </si>
+  <si>
+    <t>outdoors(garden)</t>
+  </si>
+  <si>
+    <t>household chores</t>
+  </si>
+  <si>
+    <t>house</t>
+  </si>
+  <si>
+    <t>night</t>
+  </si>
+  <si>
+    <t>Help</t>
+  </si>
+  <si>
+    <t>went on a walk together</t>
+  </si>
+  <si>
+    <t>Bonding/sport</t>
+  </si>
+  <si>
+    <t>outdoors</t>
+  </si>
+  <si>
+    <t>food(x3)</t>
   </si>
 </sst>
 </file>
@@ -339,8 +390,8 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -356,10 +407,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -679,19 +726,19 @@
         <v>5</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>54</v>
+        <v>42</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>55</v>
+        <v>43</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>56</v>
+        <v>44</v>
       </c>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.3">
@@ -702,31 +749,31 @@
         <v>46303</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>31</v>
+        <v>70</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F2" s="2">
         <v>10</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="H2" s="4" t="s">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="I2">
         <v>2</v>
       </c>
       <c r="J2" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="K2" s="7" t="s">
         <v>57</v>
-      </c>
-      <c r="K2" s="7" t="s">
-        <v>69</v>
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.3">
@@ -737,31 +784,31 @@
         <v>46304</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>9</v>
+        <v>71</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="F3" s="2">
         <v>15</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="H3" s="4" t="s">
-        <v>33</v>
+        <v>27</v>
       </c>
       <c r="I3">
         <v>10</v>
       </c>
       <c r="J3" s="7" t="s">
-        <v>58</v>
+        <v>46</v>
       </c>
       <c r="K3" s="7" t="s">
-        <v>63</v>
+        <v>51</v>
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.3">
@@ -772,28 +819,28 @@
         <v>46304</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="F4" s="2">
         <v>25</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="H4" s="4" t="s">
-        <v>33</v>
+        <v>27</v>
       </c>
       <c r="I4">
         <v>9</v>
       </c>
       <c r="J4" s="7" t="s">
-        <v>59</v>
+        <v>47</v>
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.3">
@@ -804,28 +851,28 @@
         <v>46305</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="F5" s="2">
         <v>100</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="H5" s="5" t="s">
-        <v>34</v>
+        <v>28</v>
       </c>
       <c r="I5">
         <v>10</v>
       </c>
-      <c r="J5" s="8" t="s">
-        <v>60</v>
+      <c r="J5" s="5" t="s">
+        <v>48</v>
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.3">
@@ -836,28 +883,28 @@
         <v>46305</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>16</v>
+        <v>64</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>17</v>
+        <v>67</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F6" s="2">
         <v>3</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="H6" s="5" t="s">
-        <v>34</v>
+        <v>28</v>
       </c>
       <c r="I6">
         <v>1</v>
       </c>
-      <c r="J6" s="8" t="s">
-        <v>61</v>
+      <c r="J6" s="5" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.3">
@@ -868,28 +915,28 @@
         <v>46306</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>27</v>
+        <v>72</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="F7" s="2">
         <v>180</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="H7" s="5" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="I7">
         <v>10</v>
       </c>
-      <c r="J7" s="8" t="s">
-        <v>62</v>
+      <c r="J7" s="5" t="s">
+        <v>50</v>
       </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.3">
@@ -900,28 +947,28 @@
         <v>46306</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>29</v>
+        <v>24</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="F8" s="2">
         <v>40</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="H8" s="5" t="s">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="I8">
         <v>9</v>
       </c>
-      <c r="J8" s="8" t="s">
-        <v>63</v>
+      <c r="J8" s="5" t="s">
+        <v>51</v>
       </c>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.3">
@@ -932,28 +979,28 @@
         <v>46307</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>36</v>
+        <v>63</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>37</v>
+        <v>61</v>
       </c>
       <c r="E9" s="4" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="F9" s="4">
         <v>30</v>
       </c>
       <c r="G9" s="4" t="s">
-        <v>38</v>
+        <v>30</v>
       </c>
       <c r="H9" s="5" t="s">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="I9">
         <v>10</v>
       </c>
-      <c r="J9" s="8" t="s">
-        <v>58</v>
+      <c r="J9" s="5" t="s">
+        <v>46</v>
       </c>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.3">
@@ -964,28 +1011,28 @@
         <v>46307</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>39</v>
+        <v>31</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>40</v>
+        <v>32</v>
       </c>
       <c r="E10" s="4" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="F10" s="4">
         <v>120</v>
       </c>
       <c r="G10" s="4" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="H10" s="5" t="s">
-        <v>33</v>
+        <v>27</v>
       </c>
       <c r="I10">
         <v>7</v>
       </c>
-      <c r="J10" s="8" t="s">
-        <v>64</v>
+      <c r="J10" s="5" t="s">
+        <v>52</v>
       </c>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.3">
@@ -996,28 +1043,28 @@
         <v>46308</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>41</v>
+        <v>33</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>42</v>
+        <v>73</v>
       </c>
       <c r="E11" s="4" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="F11" s="4">
         <v>40</v>
       </c>
       <c r="G11" s="4" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="H11" s="5" t="s">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="I11">
         <v>9</v>
       </c>
-      <c r="J11" s="8" t="s">
-        <v>62</v>
+      <c r="J11" s="5" t="s">
+        <v>50</v>
       </c>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.3">
@@ -1028,28 +1075,28 @@
         <v>46308</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>43</v>
+        <v>34</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>44</v>
+        <v>74</v>
       </c>
       <c r="E12" s="4" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="F12" s="4">
         <v>15</v>
       </c>
       <c r="G12" s="4" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="H12" s="5" t="s">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="I12">
         <v>3</v>
       </c>
-      <c r="J12" s="8" t="s">
-        <v>65</v>
+      <c r="J12" s="5" t="s">
+        <v>53</v>
       </c>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.3">
@@ -1060,28 +1107,28 @@
         <v>46308</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>45</v>
+        <v>35</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>46</v>
+        <v>75</v>
       </c>
       <c r="E13" s="4" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="F13" s="4">
         <v>75</v>
       </c>
       <c r="G13" s="4" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="H13" s="5" t="s">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="I13">
         <v>10</v>
       </c>
-      <c r="J13" s="8" t="s">
-        <v>66</v>
+      <c r="J13" s="5" t="s">
+        <v>54</v>
       </c>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.3">
@@ -1092,28 +1139,28 @@
         <v>46308</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>47</v>
+        <v>36</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>48</v>
+        <v>37</v>
       </c>
       <c r="E14" s="4" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="F14" s="4">
         <v>20</v>
       </c>
       <c r="G14" s="4" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="H14" s="5" t="s">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="I14">
         <v>10</v>
       </c>
-      <c r="J14" s="8" t="s">
-        <v>67</v>
+      <c r="J14" s="5" t="s">
+        <v>55</v>
       </c>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.3">
@@ -1125,28 +1172,28 @@
         <v>46309</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>49</v>
+        <v>38</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>6</v>
+        <v>76</v>
       </c>
       <c r="E15" s="4" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="F15" s="4">
         <v>7</v>
       </c>
       <c r="G15" s="4" t="s">
-        <v>50</v>
+        <v>39</v>
       </c>
       <c r="H15" s="5" t="s">
-        <v>33</v>
+        <v>27</v>
       </c>
       <c r="I15">
         <v>0</v>
       </c>
-      <c r="J15" s="8" t="s">
-        <v>68</v>
+      <c r="J15" s="5" t="s">
+        <v>56</v>
       </c>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.3">
@@ -1158,28 +1205,28 @@
         <v>46309</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>51</v>
+        <v>40</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>52</v>
+        <v>73</v>
       </c>
       <c r="E16" s="4" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="F16" s="4">
         <v>35</v>
       </c>
       <c r="G16" s="4" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="H16" s="5" t="s">
-        <v>33</v>
+        <v>27</v>
       </c>
       <c r="I16">
         <v>9</v>
       </c>
-      <c r="J16" s="8" t="s">
-        <v>63</v>
+      <c r="J16" s="5" t="s">
+        <v>51</v>
       </c>
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.3">
@@ -1191,28 +1238,28 @@
         <v>46309</v>
       </c>
       <c r="C17" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="D17" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="E17" s="4" t="s">
         <v>41</v>
-      </c>
-      <c r="D17" s="4" t="s">
-        <v>52</v>
-      </c>
-      <c r="E17" s="4" t="s">
-        <v>53</v>
       </c>
       <c r="F17" s="4">
         <v>40</v>
       </c>
       <c r="G17" s="4" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="H17" s="5" t="s">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="I17">
         <v>9</v>
       </c>
-      <c r="J17" s="8" t="s">
-        <v>59</v>
+      <c r="J17" s="5" t="s">
+        <v>47</v>
       </c>
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.3">
@@ -1223,6 +1270,27 @@
       <c r="B18" s="6">
         <v>46310</v>
       </c>
+      <c r="C18" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="D18" s="8" t="s">
+        <v>61</v>
+      </c>
+      <c r="E18" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="F18" s="8">
+        <v>130</v>
+      </c>
+      <c r="G18" s="8" t="s">
+        <v>59</v>
+      </c>
+      <c r="H18" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="I18">
+        <v>10</v>
+      </c>
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A19">
@@ -1232,6 +1300,27 @@
       <c r="B19" s="6">
         <v>46310</v>
       </c>
+      <c r="C19" s="8" t="s">
+        <v>60</v>
+      </c>
+      <c r="D19" s="8" t="s">
+        <v>77</v>
+      </c>
+      <c r="E19" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="F19" s="8">
+        <v>45</v>
+      </c>
+      <c r="G19" s="8" t="s">
+        <v>62</v>
+      </c>
+      <c r="H19" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="I19">
+        <v>10</v>
+      </c>
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A20">
@@ -1241,6 +1330,27 @@
       <c r="B20" s="6">
         <v>46310</v>
       </c>
+      <c r="C20" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="D20" s="8" t="s">
+        <v>65</v>
+      </c>
+      <c r="E20" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="F20" s="8">
+        <v>40</v>
+      </c>
+      <c r="G20" s="8" t="s">
+        <v>62</v>
+      </c>
+      <c r="H20" s="5" t="s">
+        <v>66</v>
+      </c>
+      <c r="I20">
+        <v>10</v>
+      </c>
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A21">
@@ -1248,7 +1358,28 @@
         <v>20</v>
       </c>
       <c r="B21" s="6">
-        <v>46310</v>
+        <v>46311</v>
+      </c>
+      <c r="C21" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="D21" s="8" t="s">
+        <v>82</v>
+      </c>
+      <c r="E21" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="F21" s="8">
+        <v>25</v>
+      </c>
+      <c r="G21" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="H21" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="I21">
+        <v>9</v>
       </c>
     </row>
     <row r="22" spans="1:10" x14ac:dyDescent="0.3">
@@ -1256,53 +1387,266 @@
         <f t="shared" si="0"/>
         <v>21</v>
       </c>
+      <c r="B22" s="6">
+        <v>46311</v>
+      </c>
+      <c r="C22" s="8" t="s">
+        <v>83</v>
+      </c>
+      <c r="D22" s="8" t="s">
+        <v>84</v>
+      </c>
+      <c r="E22" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="F22" s="8">
+        <v>100</v>
+      </c>
+      <c r="G22" s="8" t="s">
+        <v>85</v>
+      </c>
+      <c r="H22" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="I22">
+        <v>10</v>
+      </c>
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A23">
         <f t="shared" si="0"/>
         <v>22</v>
       </c>
+      <c r="B23" s="6">
+        <v>46311</v>
+      </c>
+      <c r="C23" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="D23" s="8" t="s">
+        <v>73</v>
+      </c>
+      <c r="E23" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="F23" s="8">
+        <v>45</v>
+      </c>
+      <c r="G23" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="H23" s="5" t="s">
+        <v>81</v>
+      </c>
+      <c r="I23">
+        <v>10</v>
+      </c>
     </row>
     <row r="24" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A24">
         <f t="shared" si="0"/>
         <v>23</v>
       </c>
+      <c r="B24" s="6">
+        <v>46312</v>
+      </c>
+      <c r="C24" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="D24" s="8" t="s">
+        <v>68</v>
+      </c>
+      <c r="E24" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="F24" s="8">
+        <v>30</v>
+      </c>
+      <c r="G24" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="H24" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="I24">
+        <v>7</v>
+      </c>
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A25">
         <f t="shared" si="0"/>
         <v>24</v>
       </c>
+      <c r="B25" s="6">
+        <v>46312</v>
+      </c>
+      <c r="C25" s="8" t="s">
+        <v>69</v>
+      </c>
+      <c r="D25" s="8" t="s">
+        <v>72</v>
+      </c>
+      <c r="E25" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="F25" s="8">
+        <v>120</v>
+      </c>
+      <c r="G25" s="8" t="s">
+        <v>78</v>
+      </c>
+      <c r="H25" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="I25">
+        <v>8</v>
+      </c>
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A26">
         <f t="shared" si="0"/>
         <v>25</v>
       </c>
+      <c r="B26" s="6">
+        <v>46312</v>
+      </c>
+      <c r="C26" s="8" t="s">
+        <v>79</v>
+      </c>
+      <c r="D26" s="8" t="s">
+        <v>32</v>
+      </c>
+      <c r="E26" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="F26" s="8">
+        <v>30</v>
+      </c>
+      <c r="G26" s="8" t="s">
+        <v>80</v>
+      </c>
+      <c r="H26" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="I26">
+        <v>6</v>
+      </c>
     </row>
     <row r="27" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A27">
         <f t="shared" si="0"/>
         <v>26</v>
       </c>
+      <c r="B27" s="6">
+        <v>46312</v>
+      </c>
+      <c r="C27" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="D27" s="8" t="s">
+        <v>73</v>
+      </c>
+      <c r="E27" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="F27" s="8">
+        <v>40</v>
+      </c>
+      <c r="G27" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="H27" s="5" t="s">
+        <v>81</v>
+      </c>
     </row>
     <row r="28" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A28">
         <f t="shared" si="0"/>
         <v>27</v>
       </c>
+      <c r="B28" s="6">
+        <v>46313</v>
+      </c>
+      <c r="C28" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="D28" s="8" t="s">
+        <v>72</v>
+      </c>
+      <c r="E28" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="F28" s="8">
+        <v>195</v>
+      </c>
+      <c r="G28" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="H28" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="I28">
+        <v>10</v>
+      </c>
     </row>
     <row r="29" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A29">
         <f t="shared" si="0"/>
         <v>28</v>
       </c>
+      <c r="B29" s="6">
+        <v>46313</v>
+      </c>
+      <c r="C29" s="8" t="s">
+        <v>79</v>
+      </c>
+      <c r="D29" s="8" t="s">
+        <v>82</v>
+      </c>
+      <c r="E29" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="F29" s="8">
+        <v>40</v>
+      </c>
+      <c r="G29" s="8" t="s">
+        <v>80</v>
+      </c>
+      <c r="H29" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="I29">
+        <v>5</v>
+      </c>
     </row>
     <row r="30" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A30">
         <f t="shared" si="0"/>
         <v>29</v>
+      </c>
+      <c r="B30" s="6">
+        <v>46313</v>
+      </c>
+      <c r="C30" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="D30" s="8" t="s">
+        <v>86</v>
+      </c>
+      <c r="E30" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="F30" s="8">
+        <v>35</v>
+      </c>
+      <c r="G30" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="H30" s="5" t="s">
+        <v>81</v>
+      </c>
+      <c r="I30">
+        <v>10</v>
       </c>
     </row>
     <row r="31" spans="1:10" x14ac:dyDescent="0.3">
@@ -1437,9 +1781,12 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1587,26 +1934,15 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B15FDCE2-C38D-4DD1-B711-A8CB81A27211}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{33023472-F23D-4624-BC7A-4AE1438DE3EC}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="75eb23ce-bee3-4614-ac9d-e7493ba98713"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -1630,9 +1966,17 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{33023472-F23D-4624-BC7A-4AE1438DE3EC}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B15FDCE2-C38D-4DD1-B711-A8CB81A27211}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="75eb23ce-bee3-4614-ac9d-e7493ba98713"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Flower design prototype + data points added
</commit_message>
<xml_diff>
--- a/Dear_Data_Project/sibling_data.xlsx
+++ b/Dear_Data_Project/sibling_data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/4072360cc263ec0b/Processing/DearDataProject/Dear Data Project/Dear_Data_Project/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="205" documentId="8_{F06C03BE-BA34-4718-934D-620FB05A1E63}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B25BE202-2DB5-4D1C-B1FC-0CB240600BDF}"/>
+  <xr:revisionPtr revIDLastSave="304" documentId="8_{F06C03BE-BA34-4718-934D-620FB05A1E63}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C22DAA21-0149-44B6-AAF9-40A275FEA1C7}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="174" uniqueCount="87">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="249" uniqueCount="96">
   <si>
     <t>ID</t>
   </si>
@@ -294,6 +294,33 @@
   </si>
   <si>
     <t>food(x3)</t>
+  </si>
+  <si>
+    <t>annoyed</t>
+  </si>
+  <si>
+    <t>neutral</t>
+  </si>
+  <si>
+    <t>tired</t>
+  </si>
+  <si>
+    <t>enerdised</t>
+  </si>
+  <si>
+    <t>sleepy</t>
+  </si>
+  <si>
+    <t>bored</t>
+  </si>
+  <si>
+    <t>made a snack together</t>
+  </si>
+  <si>
+    <t>Shared activity/food</t>
+  </si>
+  <si>
+    <t>Entertainment/food</t>
   </si>
 </sst>
 </file>
@@ -407,6 +434,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -842,6 +873,9 @@
       <c r="J4" s="7" t="s">
         <v>47</v>
       </c>
+      <c r="K4" s="7" t="s">
+        <v>51</v>
+      </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A5" s="2">
@@ -874,6 +908,9 @@
       <c r="J5" s="5" t="s">
         <v>48</v>
       </c>
+      <c r="K5" s="5" t="s">
+        <v>48</v>
+      </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A6" s="2">
@@ -906,6 +943,9 @@
       <c r="J6" s="5" t="s">
         <v>49</v>
       </c>
+      <c r="K6" s="5" t="s">
+        <v>87</v>
+      </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A7" s="2">
@@ -938,6 +978,9 @@
       <c r="J7" s="5" t="s">
         <v>50</v>
       </c>
+      <c r="K7" s="5" t="s">
+        <v>48</v>
+      </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A8" s="2">
@@ -970,6 +1013,9 @@
       <c r="J8" s="5" t="s">
         <v>51</v>
       </c>
+      <c r="K8" s="5" t="s">
+        <v>88</v>
+      </c>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A9" s="4">
@@ -1002,6 +1048,9 @@
       <c r="J9" s="5" t="s">
         <v>46</v>
       </c>
+      <c r="K9" s="5" t="s">
+        <v>51</v>
+      </c>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A10" s="4">
@@ -1034,6 +1083,9 @@
       <c r="J10" s="5" t="s">
         <v>52</v>
       </c>
+      <c r="K10" s="5" t="s">
+        <v>89</v>
+      </c>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A11" s="4">
@@ -1066,6 +1118,9 @@
       <c r="J11" s="5" t="s">
         <v>50</v>
       </c>
+      <c r="K11" s="5" t="s">
+        <v>90</v>
+      </c>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A12" s="4">
@@ -1098,6 +1153,9 @@
       <c r="J12" s="5" t="s">
         <v>53</v>
       </c>
+      <c r="K12" s="5" t="s">
+        <v>57</v>
+      </c>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A13" s="4">
@@ -1130,6 +1188,9 @@
       <c r="J13" s="5" t="s">
         <v>54</v>
       </c>
+      <c r="K13" s="5" t="s">
+        <v>48</v>
+      </c>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A14" s="4">
@@ -1161,6 +1222,9 @@
       </c>
       <c r="J14" s="5" t="s">
         <v>55</v>
+      </c>
+      <c r="K14" s="5" t="s">
+        <v>91</v>
       </c>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.3">
@@ -1195,6 +1259,9 @@
       <c r="J15" s="5" t="s">
         <v>56</v>
       </c>
+      <c r="K15" s="5" t="s">
+        <v>53</v>
+      </c>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A16">
@@ -1228,8 +1295,11 @@
       <c r="J16" s="5" t="s">
         <v>51</v>
       </c>
-    </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K16" s="5" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A17">
         <f t="shared" si="0"/>
         <v>16</v>
@@ -1261,8 +1331,11 @@
       <c r="J17" s="5" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K17" s="5" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A18">
         <f t="shared" si="0"/>
         <v>17</v>
@@ -1270,19 +1343,19 @@
       <c r="B18" s="6">
         <v>46310</v>
       </c>
-      <c r="C18" s="8" t="s">
+      <c r="C18" s="4" t="s">
         <v>58</v>
       </c>
-      <c r="D18" s="8" t="s">
+      <c r="D18" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="E18" s="8" t="s">
+      <c r="E18" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="F18" s="8">
+      <c r="F18" s="4">
         <v>130</v>
       </c>
-      <c r="G18" s="8" t="s">
+      <c r="G18" s="4" t="s">
         <v>59</v>
       </c>
       <c r="H18" s="5" t="s">
@@ -1291,8 +1364,14 @@
       <c r="I18">
         <v>10</v>
       </c>
-    </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="J18" s="5" t="s">
+        <v>92</v>
+      </c>
+      <c r="K18" s="5" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="19" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A19">
         <f t="shared" si="0"/>
         <v>18</v>
@@ -1300,19 +1379,19 @@
       <c r="B19" s="6">
         <v>46310</v>
       </c>
-      <c r="C19" s="8" t="s">
+      <c r="C19" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="D19" s="8" t="s">
+      <c r="D19" s="4" t="s">
         <v>77</v>
       </c>
-      <c r="E19" s="8" t="s">
+      <c r="E19" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="F19" s="8">
+      <c r="F19" s="4">
         <v>45</v>
       </c>
-      <c r="G19" s="8" t="s">
+      <c r="G19" s="4" t="s">
         <v>62</v>
       </c>
       <c r="H19" s="5" t="s">
@@ -1321,8 +1400,14 @@
       <c r="I19">
         <v>10</v>
       </c>
-    </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="J19" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="K19" s="5" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="20" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A20">
         <f t="shared" si="0"/>
         <v>19</v>
@@ -1330,19 +1415,19 @@
       <c r="B20" s="6">
         <v>46310</v>
       </c>
-      <c r="C20" s="8" t="s">
+      <c r="C20" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="D20" s="8" t="s">
+      <c r="D20" s="4" t="s">
         <v>65</v>
       </c>
-      <c r="E20" s="8" t="s">
+      <c r="E20" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="F20" s="8">
+      <c r="F20" s="4">
         <v>40</v>
       </c>
-      <c r="G20" s="8" t="s">
+      <c r="G20" s="4" t="s">
         <v>62</v>
       </c>
       <c r="H20" s="5" t="s">
@@ -1351,8 +1436,14 @@
       <c r="I20">
         <v>10</v>
       </c>
-    </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="J20" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="K20" s="5" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="21" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A21">
         <f t="shared" si="0"/>
         <v>20</v>
@@ -1360,19 +1451,19 @@
       <c r="B21" s="6">
         <v>46311</v>
       </c>
-      <c r="C21" s="8" t="s">
+      <c r="C21" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="D21" s="8" t="s">
+      <c r="D21" s="4" t="s">
         <v>82</v>
       </c>
-      <c r="E21" s="8" t="s">
+      <c r="E21" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="F21" s="8">
+      <c r="F21" s="4">
         <v>25</v>
       </c>
-      <c r="G21" s="8" t="s">
+      <c r="G21" s="4" t="s">
         <v>19</v>
       </c>
       <c r="H21" s="5" t="s">
@@ -1381,8 +1472,14 @@
       <c r="I21">
         <v>9</v>
       </c>
-    </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="J21" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="K21" s="5" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="22" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A22">
         <f t="shared" si="0"/>
         <v>21</v>
@@ -1390,19 +1487,19 @@
       <c r="B22" s="6">
         <v>46311</v>
       </c>
-      <c r="C22" s="8" t="s">
+      <c r="C22" s="4" t="s">
         <v>83</v>
       </c>
-      <c r="D22" s="8" t="s">
+      <c r="D22" s="4" t="s">
         <v>84</v>
       </c>
-      <c r="E22" s="8" t="s">
+      <c r="E22" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="F22" s="8">
+      <c r="F22" s="4">
         <v>100</v>
       </c>
-      <c r="G22" s="8" t="s">
+      <c r="G22" s="4" t="s">
         <v>85</v>
       </c>
       <c r="H22" s="5" t="s">
@@ -1411,8 +1508,14 @@
       <c r="I22">
         <v>10</v>
       </c>
-    </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="J22" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="K22" s="5" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="23" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A23">
         <f t="shared" si="0"/>
         <v>22</v>
@@ -1420,19 +1523,19 @@
       <c r="B23" s="6">
         <v>46311</v>
       </c>
-      <c r="C23" s="8" t="s">
+      <c r="C23" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="D23" s="8" t="s">
+      <c r="D23" s="4" t="s">
         <v>73</v>
       </c>
-      <c r="E23" s="8" t="s">
+      <c r="E23" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="F23" s="8">
+      <c r="F23" s="4">
         <v>45</v>
       </c>
-      <c r="G23" s="8" t="s">
+      <c r="G23" s="4" t="s">
         <v>11</v>
       </c>
       <c r="H23" s="5" t="s">
@@ -1441,8 +1544,14 @@
       <c r="I23">
         <v>10</v>
       </c>
-    </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="J23" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="K23" s="5" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="24" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A24">
         <f t="shared" si="0"/>
         <v>23</v>
@@ -1450,19 +1559,19 @@
       <c r="B24" s="6">
         <v>46312</v>
       </c>
-      <c r="C24" s="8" t="s">
+      <c r="C24" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="D24" s="8" t="s">
+      <c r="D24" s="4" t="s">
         <v>68</v>
       </c>
-      <c r="E24" s="8" t="s">
+      <c r="E24" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="F24" s="8">
+      <c r="F24" s="4">
         <v>30</v>
       </c>
-      <c r="G24" s="8" t="s">
+      <c r="G24" s="4" t="s">
         <v>14</v>
       </c>
       <c r="H24" s="5" t="s">
@@ -1471,8 +1580,14 @@
       <c r="I24">
         <v>7</v>
       </c>
-    </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="J24" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="K24" s="5" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="25" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A25">
         <f t="shared" si="0"/>
         <v>24</v>
@@ -1480,19 +1595,19 @@
       <c r="B25" s="6">
         <v>46312</v>
       </c>
-      <c r="C25" s="8" t="s">
+      <c r="C25" s="4" t="s">
         <v>69</v>
       </c>
-      <c r="D25" s="8" t="s">
+      <c r="D25" s="4" t="s">
         <v>72</v>
       </c>
-      <c r="E25" s="8" t="s">
+      <c r="E25" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="F25" s="8">
+      <c r="F25" s="4">
         <v>120</v>
       </c>
-      <c r="G25" s="8" t="s">
+      <c r="G25" s="4" t="s">
         <v>78</v>
       </c>
       <c r="H25" s="5" t="s">
@@ -1501,8 +1616,14 @@
       <c r="I25">
         <v>8</v>
       </c>
-    </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="J25" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="K25" s="5" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="26" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A26">
         <f t="shared" si="0"/>
         <v>25</v>
@@ -1510,19 +1631,19 @@
       <c r="B26" s="6">
         <v>46312</v>
       </c>
-      <c r="C26" s="8" t="s">
+      <c r="C26" s="4" t="s">
         <v>79</v>
       </c>
-      <c r="D26" s="8" t="s">
+      <c r="D26" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="E26" s="8" t="s">
+      <c r="E26" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="F26" s="8">
+      <c r="F26" s="4">
         <v>30</v>
       </c>
-      <c r="G26" s="8" t="s">
+      <c r="G26" s="4" t="s">
         <v>80</v>
       </c>
       <c r="H26" s="5" t="s">
@@ -1531,8 +1652,14 @@
       <c r="I26">
         <v>6</v>
       </c>
-    </row>
-    <row r="27" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="J26" s="5" t="s">
+        <v>87</v>
+      </c>
+      <c r="K26" s="5" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="27" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A27">
         <f t="shared" si="0"/>
         <v>26</v>
@@ -1540,26 +1667,32 @@
       <c r="B27" s="6">
         <v>46312</v>
       </c>
-      <c r="C27" s="8" t="s">
+      <c r="C27" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="D27" s="8" t="s">
+      <c r="D27" s="4" t="s">
         <v>73</v>
       </c>
-      <c r="E27" s="8" t="s">
+      <c r="E27" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="F27" s="8">
+      <c r="F27" s="4">
         <v>40</v>
       </c>
-      <c r="G27" s="8" t="s">
+      <c r="G27" s="4" t="s">
         <v>11</v>
       </c>
       <c r="H27" s="5" t="s">
         <v>81</v>
       </c>
-    </row>
-    <row r="28" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="J27" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="K27" s="5" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="28" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A28">
         <f t="shared" si="0"/>
         <v>27</v>
@@ -1567,19 +1700,19 @@
       <c r="B28" s="6">
         <v>46313</v>
       </c>
-      <c r="C28" s="8" t="s">
+      <c r="C28" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="D28" s="8" t="s">
+      <c r="D28" s="4" t="s">
         <v>72</v>
       </c>
-      <c r="E28" s="8" t="s">
+      <c r="E28" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="F28" s="8">
+      <c r="F28" s="4">
         <v>195</v>
       </c>
-      <c r="G28" s="8" t="s">
+      <c r="G28" s="4" t="s">
         <v>22</v>
       </c>
       <c r="H28" s="5" t="s">
@@ -1588,8 +1721,14 @@
       <c r="I28">
         <v>10</v>
       </c>
-    </row>
-    <row r="29" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="J28" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="K28" s="5" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="29" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A29">
         <f t="shared" si="0"/>
         <v>28</v>
@@ -1597,19 +1736,19 @@
       <c r="B29" s="6">
         <v>46313</v>
       </c>
-      <c r="C29" s="8" t="s">
+      <c r="C29" s="4" t="s">
         <v>79</v>
       </c>
-      <c r="D29" s="8" t="s">
+      <c r="D29" s="4" t="s">
         <v>82</v>
       </c>
-      <c r="E29" s="8" t="s">
+      <c r="E29" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="F29" s="8">
+      <c r="F29" s="4">
         <v>40</v>
       </c>
-      <c r="G29" s="8" t="s">
+      <c r="G29" s="4" t="s">
         <v>80</v>
       </c>
       <c r="H29" s="5" t="s">
@@ -1618,8 +1757,14 @@
       <c r="I29">
         <v>5</v>
       </c>
-    </row>
-    <row r="30" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="J29" s="5" t="s">
+        <v>87</v>
+      </c>
+      <c r="K29" s="5" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="30" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A30">
         <f t="shared" si="0"/>
         <v>29</v>
@@ -1627,19 +1772,19 @@
       <c r="B30" s="6">
         <v>46313</v>
       </c>
-      <c r="C30" s="8" t="s">
+      <c r="C30" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="D30" s="8" t="s">
+      <c r="D30" s="4" t="s">
         <v>86</v>
       </c>
-      <c r="E30" s="8" t="s">
+      <c r="E30" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="F30" s="8">
+      <c r="F30" s="4">
         <v>35</v>
       </c>
-      <c r="G30" s="8" t="s">
+      <c r="G30" s="4" t="s">
         <v>11</v>
       </c>
       <c r="H30" s="5" t="s">
@@ -1648,110 +1793,266 @@
       <c r="I30">
         <v>10</v>
       </c>
-    </row>
-    <row r="31" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="J30" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="K30" s="5" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="31" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A31">
         <f t="shared" si="0"/>
         <v>30</v>
       </c>
-    </row>
-    <row r="32" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="B31" s="6">
+        <v>46314</v>
+      </c>
+      <c r="C31" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="D31" s="8" t="s">
+        <v>82</v>
+      </c>
+      <c r="E31" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="F31" s="8">
+        <v>20</v>
+      </c>
+      <c r="G31" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="H31" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="I31">
+        <v>9</v>
+      </c>
+      <c r="J31" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="K31" s="5" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="32" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A32">
         <f t="shared" si="0"/>
         <v>31</v>
       </c>
-    </row>
-    <row r="33" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B32" s="6">
+        <v>46314</v>
+      </c>
+      <c r="C32" s="8" t="s">
+        <v>93</v>
+      </c>
+      <c r="D32" s="8" t="s">
+        <v>94</v>
+      </c>
+      <c r="E32" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="F32" s="8">
+        <v>15</v>
+      </c>
+      <c r="G32" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="H32" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="I32">
+        <v>10</v>
+      </c>
+      <c r="J32" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="K32" s="5" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="33" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A33">
         <f t="shared" si="0"/>
         <v>32</v>
       </c>
-    </row>
-    <row r="34" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B33" s="6">
+        <v>46314</v>
+      </c>
+      <c r="C33" s="8" t="s">
+        <v>63</v>
+      </c>
+      <c r="D33" s="8" t="s">
+        <v>95</v>
+      </c>
+      <c r="E33" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="F33" s="8">
+        <v>45</v>
+      </c>
+      <c r="G33" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="H33" s="5" t="s">
+        <v>81</v>
+      </c>
+      <c r="I33">
+        <v>10</v>
+      </c>
+      <c r="J33" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="K33" s="5" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="34" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A34">
         <f t="shared" si="0"/>
         <v>33</v>
       </c>
-    </row>
-    <row r="35" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B34" s="6">
+        <v>46314</v>
+      </c>
+      <c r="C34" s="8" t="s">
+        <v>79</v>
+      </c>
+      <c r="D34" s="8" t="s">
+        <v>82</v>
+      </c>
+      <c r="E34" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="F34" s="8">
+        <v>20</v>
+      </c>
+      <c r="G34" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="H34" s="5" t="s">
+        <v>81</v>
+      </c>
+      <c r="I34">
+        <v>4</v>
+      </c>
+      <c r="J34" s="5" t="s">
+        <v>89</v>
+      </c>
+      <c r="K34" s="5" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="35" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A35">
         <f t="shared" si="0"/>
         <v>34</v>
       </c>
-    </row>
-    <row r="36" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B35" s="6">
+        <v>46314</v>
+      </c>
+      <c r="C35" s="8" t="s">
+        <v>36</v>
+      </c>
+      <c r="D35" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="E35" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="F35" s="8">
+        <v>15</v>
+      </c>
+      <c r="G35" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="H35" s="5" t="s">
+        <v>81</v>
+      </c>
+      <c r="I35">
+        <v>10</v>
+      </c>
+      <c r="J35" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="K35" s="5" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="36" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A36">
         <f t="shared" si="0"/>
         <v>35</v>
       </c>
     </row>
-    <row r="37" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A37">
         <f t="shared" si="0"/>
         <v>36</v>
       </c>
     </row>
-    <row r="38" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A38">
         <f t="shared" si="0"/>
         <v>37</v>
       </c>
     </row>
-    <row r="39" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A39">
         <f t="shared" si="0"/>
         <v>38</v>
       </c>
     </row>
-    <row r="40" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A40">
         <f t="shared" si="0"/>
         <v>39</v>
       </c>
     </row>
-    <row r="41" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A41">
         <f t="shared" si="0"/>
         <v>40</v>
       </c>
     </row>
-    <row r="42" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A42">
         <f t="shared" si="0"/>
         <v>41</v>
       </c>
     </row>
-    <row r="43" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A43">
         <f t="shared" si="0"/>
         <v>42</v>
       </c>
     </row>
-    <row r="44" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A44">
         <f t="shared" si="0"/>
         <v>43</v>
       </c>
     </row>
-    <row r="45" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A45">
         <f t="shared" si="0"/>
         <v>44</v>
       </c>
     </row>
-    <row r="46" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A46">
         <f t="shared" si="0"/>
         <v>45</v>
       </c>
     </row>
-    <row r="47" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A47">
         <f t="shared" si="0"/>
         <v>46</v>
       </c>
     </row>
-    <row r="48" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A48">
         <f t="shared" si="0"/>
         <v>47</v>
@@ -1781,6 +2082,12 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
@@ -1789,7 +2096,7 @@
 </FormTemplates>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100E802F14A90D1B345818A6FFB06D8A03D" ma:contentTypeVersion="4" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ea7226ff09ef22af6f5ba21dc65cff36">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="75eb23ce-bee3-4614-ac9d-e7493ba98713" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="807d9844cc6c643302a5e086dcc98a76" ns3:_="">
     <xsd:import namespace="75eb23ce-bee3-4614-ac9d-e7493ba98713"/>
@@ -1933,13 +2240,23 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B15FDCE2-C38D-4DD1-B711-A8CB81A27211}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="75eb23ce-bee3-4614-ac9d-e7493ba98713"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{33023472-F23D-4624-BC7A-4AE1438DE3EC}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
@@ -1947,7 +2264,7 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{997A7A74-A1F7-48AE-82CD-9856C622E446}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1963,20 +2280,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B15FDCE2-C38D-4DD1-B711-A8CB81A27211}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="75eb23ce-bee3-4614-ac9d-e7493ba98713"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
ideas for shapes and more data points
</commit_message>
<xml_diff>
--- a/Dear_Data_Project/sibling_data.xlsx
+++ b/Dear_Data_Project/sibling_data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/4072360cc263ec0b/Processing/DearDataProject/Dear Data Project/Dear_Data_Project/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="395" documentId="8_{F06C03BE-BA34-4718-934D-620FB05A1E63}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{02028AF9-B72D-4432-A793-24CEED22EB1A}"/>
+  <xr:revisionPtr revIDLastSave="665" documentId="8_{F06C03BE-BA34-4718-934D-620FB05A1E63}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{053BE4D8-43B8-457A-9F12-E03959E7E185}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="305" uniqueCount="103">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="480" uniqueCount="118">
   <si>
     <t>ID</t>
   </si>
@@ -342,6 +342,51 @@
   </si>
   <si>
     <t>satisfied</t>
+  </si>
+  <si>
+    <t>me</t>
+  </si>
+  <si>
+    <t>watched movie together</t>
+  </si>
+  <si>
+    <t xml:space="preserve">went grocery shopping </t>
+  </si>
+  <si>
+    <t>outdoors(tesco)</t>
+  </si>
+  <si>
+    <t>food (x2)</t>
+  </si>
+  <si>
+    <t>picked from school(rainy)</t>
+  </si>
+  <si>
+    <t>entertainment</t>
+  </si>
+  <si>
+    <t>help</t>
+  </si>
+  <si>
+    <t>dropped at dance class</t>
+  </si>
+  <si>
+    <t>bonding</t>
+  </si>
+  <si>
+    <t>made breakfast for my sister</t>
+  </si>
+  <si>
+    <t>made lunch together</t>
+  </si>
+  <si>
+    <t>cleaned house together</t>
+  </si>
+  <si>
+    <t>food *2</t>
+  </si>
+  <si>
+    <t>food*3</t>
   </si>
 </sst>
 </file>
@@ -428,7 +473,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -440,6 +485,7 @@
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -746,7 +792,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K51"/>
+  <dimension ref="A1:K71"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -1286,7 +1332,7 @@
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A16">
-        <f t="shared" ref="A16:A51" si="0">SUM(A15,1)</f>
+        <f t="shared" ref="A16:A56" si="0">SUM(A15,1)</f>
         <v>15</v>
       </c>
       <c r="B16" s="6">
@@ -2009,19 +2055,19 @@
       <c r="B36" s="6">
         <v>46315</v>
       </c>
-      <c r="C36" s="8" t="s">
+      <c r="C36" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="D36" s="8" t="s">
+      <c r="D36" s="4" t="s">
         <v>82</v>
       </c>
-      <c r="E36" s="8" t="s">
+      <c r="E36" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="F36" s="8">
+      <c r="F36" s="4">
         <v>25</v>
       </c>
-      <c r="G36" s="8" t="s">
+      <c r="G36" s="4" t="s">
         <v>19</v>
       </c>
       <c r="H36" s="5" t="s">
@@ -2045,19 +2091,19 @@
       <c r="B37" s="6">
         <v>46315</v>
       </c>
-      <c r="C37" s="8" t="s">
+      <c r="C37" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="D37" s="8" t="s">
+      <c r="D37" s="4" t="s">
         <v>96</v>
       </c>
-      <c r="E37" s="8" t="s">
-        <v>13</v>
-      </c>
-      <c r="F37" s="8">
+      <c r="E37" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F37" s="4">
         <v>60</v>
       </c>
-      <c r="G37" s="8" t="s">
+      <c r="G37" s="4" t="s">
         <v>11</v>
       </c>
       <c r="H37" s="5" t="s">
@@ -2081,19 +2127,19 @@
       <c r="B38" s="6">
         <v>46315</v>
       </c>
-      <c r="C38" s="8" t="s">
+      <c r="C38" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="D38" s="8" t="s">
+      <c r="D38" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="E38" s="8" t="s">
-        <v>13</v>
-      </c>
-      <c r="F38" s="8">
+      <c r="E38" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F38" s="4">
         <v>60</v>
       </c>
-      <c r="G38" s="8" t="s">
+      <c r="G38" s="4" t="s">
         <v>7</v>
       </c>
       <c r="H38" s="5" t="s">
@@ -2117,19 +2163,19 @@
       <c r="B39" s="6">
         <v>46315</v>
       </c>
-      <c r="C39" s="8" t="s">
+      <c r="C39" s="4" t="s">
         <v>97</v>
       </c>
-      <c r="D39" s="8" t="s">
+      <c r="D39" s="4" t="s">
         <v>99</v>
       </c>
-      <c r="E39" s="8" t="s">
+      <c r="E39" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="F39" s="8">
+      <c r="F39" s="4">
         <v>30</v>
       </c>
-      <c r="G39" s="8" t="s">
+      <c r="G39" s="4" t="s">
         <v>7</v>
       </c>
       <c r="H39" s="5" t="s">
@@ -2153,19 +2199,19 @@
       <c r="B40" s="6">
         <v>46315</v>
       </c>
-      <c r="C40" s="8" t="s">
+      <c r="C40" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="D40" s="8" t="s">
+      <c r="D40" s="4" t="s">
         <v>73</v>
       </c>
-      <c r="E40" s="8" t="s">
-        <v>13</v>
-      </c>
-      <c r="F40" s="8">
+      <c r="E40" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F40" s="4">
         <v>45</v>
       </c>
-      <c r="G40" s="8" t="s">
+      <c r="G40" s="4" t="s">
         <v>11</v>
       </c>
       <c r="H40" s="5" t="s">
@@ -2189,19 +2235,19 @@
       <c r="B41" s="6">
         <v>46316</v>
       </c>
-      <c r="C41" s="8" t="s">
+      <c r="C41" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="D41" s="8" t="s">
+      <c r="D41" s="4" t="s">
         <v>82</v>
       </c>
-      <c r="E41" s="8" t="s">
+      <c r="E41" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="F41" s="8">
+      <c r="F41" s="4">
         <v>25</v>
       </c>
-      <c r="G41" s="8" t="s">
+      <c r="G41" s="4" t="s">
         <v>19</v>
       </c>
       <c r="H41" s="5" t="s">
@@ -2225,19 +2271,19 @@
       <c r="B42" s="6">
         <v>46316</v>
       </c>
-      <c r="C42" s="8" t="s">
+      <c r="C42" s="4" t="s">
         <v>101</v>
       </c>
-      <c r="D42" s="8" t="s">
+      <c r="D42" s="4" t="s">
         <v>100</v>
       </c>
-      <c r="E42" s="8" t="s">
+      <c r="E42" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="F42" s="8">
+      <c r="F42" s="4">
         <v>30</v>
       </c>
-      <c r="G42" s="8" t="s">
+      <c r="G42" s="4" t="s">
         <v>14</v>
       </c>
       <c r="H42" s="5" t="s">
@@ -2261,19 +2307,19 @@
       <c r="B43" s="6">
         <v>46316</v>
       </c>
-      <c r="C43" s="8" t="s">
+      <c r="C43" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="D43" s="8" t="s">
+      <c r="D43" s="4" t="s">
         <v>73</v>
       </c>
-      <c r="E43" s="8" t="s">
-        <v>13</v>
-      </c>
-      <c r="F43" s="8">
+      <c r="E43" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F43" s="4">
         <v>45</v>
       </c>
-      <c r="G43" s="8" t="s">
+      <c r="G43" s="4" t="s">
         <v>11</v>
       </c>
       <c r="H43" s="5" t="s">
@@ -2294,47 +2340,917 @@
         <f t="shared" si="0"/>
         <v>43</v>
       </c>
+      <c r="B44" s="6">
+        <v>46317</v>
+      </c>
+      <c r="C44" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="D44" s="4" t="s">
+        <v>82</v>
+      </c>
+      <c r="E44" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="F44" s="4">
+        <v>25</v>
+      </c>
+      <c r="G44" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="H44" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="I44">
+        <v>10</v>
+      </c>
+      <c r="J44" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="K44" s="5" t="s">
+        <v>50</v>
+      </c>
     </row>
     <row r="45" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A45">
         <f t="shared" si="0"/>
         <v>44</v>
       </c>
+      <c r="B45" s="6">
+        <v>46317</v>
+      </c>
+      <c r="C45" s="4" t="s">
+        <v>104</v>
+      </c>
+      <c r="D45" s="4" t="s">
+        <v>109</v>
+      </c>
+      <c r="E45" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F45" s="4">
+        <v>120</v>
+      </c>
+      <c r="G45" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="H45" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="I45">
+        <v>10</v>
+      </c>
+      <c r="J45" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="K45" s="5" t="s">
+        <v>51</v>
+      </c>
     </row>
     <row r="46" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A46">
         <f t="shared" si="0"/>
         <v>45</v>
       </c>
+      <c r="B46" s="6">
+        <v>46317</v>
+      </c>
+      <c r="C46" s="4" t="s">
+        <v>105</v>
+      </c>
+      <c r="D46" s="4" t="s">
+        <v>110</v>
+      </c>
+      <c r="E46" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F46" s="4">
+        <v>125</v>
+      </c>
+      <c r="G46" s="4" t="s">
+        <v>106</v>
+      </c>
+      <c r="H46" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="I46">
+        <v>10</v>
+      </c>
+      <c r="J46" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="K46" s="5" t="s">
+        <v>47</v>
+      </c>
     </row>
     <row r="47" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A47">
         <f t="shared" si="0"/>
         <v>46</v>
       </c>
+      <c r="B47" s="6">
+        <v>46317</v>
+      </c>
+      <c r="C47" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="D47" s="4" t="s">
+        <v>107</v>
+      </c>
+      <c r="E47" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F47" s="4">
+        <v>40</v>
+      </c>
+      <c r="G47" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="H47" s="5" t="s">
+        <v>81</v>
+      </c>
+      <c r="I47">
+        <v>10</v>
+      </c>
+      <c r="J47" s="5" t="s">
+        <v>102</v>
+      </c>
+      <c r="K47" s="5" t="s">
+        <v>102</v>
+      </c>
     </row>
     <row r="48" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A48">
         <f t="shared" si="0"/>
         <v>47</v>
       </c>
-    </row>
-    <row r="49" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B48" s="6">
+        <v>46318</v>
+      </c>
+      <c r="C48" s="4" t="s">
+        <v>108</v>
+      </c>
+      <c r="D48" s="4" t="s">
+        <v>82</v>
+      </c>
+      <c r="E48" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="F48" s="4">
+        <v>20</v>
+      </c>
+      <c r="G48" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="H48" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="I48">
+        <v>6</v>
+      </c>
+      <c r="J48" s="5" t="s">
+        <v>87</v>
+      </c>
+      <c r="K48" s="5" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="49" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A49">
         <f t="shared" si="0"/>
         <v>48</v>
       </c>
-    </row>
-    <row r="50" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B49" s="6">
+        <v>46318</v>
+      </c>
+      <c r="C49" s="4" t="s">
+        <v>111</v>
+      </c>
+      <c r="D49" s="4" t="s">
+        <v>110</v>
+      </c>
+      <c r="E49" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="F49" s="4">
+        <v>10</v>
+      </c>
+      <c r="G49" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="H49" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="I49">
+        <v>8</v>
+      </c>
+      <c r="J49" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="K49" s="5" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="50" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A50">
         <f t="shared" si="0"/>
         <v>49</v>
       </c>
-    </row>
-    <row r="51" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B50" s="6">
+        <v>46318</v>
+      </c>
+      <c r="C50" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="D50" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="E50" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F50" s="4">
+        <v>30</v>
+      </c>
+      <c r="G50" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="H50" s="5" t="s">
+        <v>81</v>
+      </c>
+      <c r="I50">
+        <v>10</v>
+      </c>
+      <c r="J50" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="K50" s="5" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="51" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A51">
         <f t="shared" si="0"/>
         <v>50</v>
+      </c>
+      <c r="B51" s="6">
+        <v>46318</v>
+      </c>
+      <c r="C51" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="D51" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="E51" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F51" s="4">
+        <v>40</v>
+      </c>
+      <c r="G51" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="H51" s="5" t="s">
+        <v>81</v>
+      </c>
+      <c r="I51">
+        <v>10</v>
+      </c>
+      <c r="J51" s="5" t="s">
+        <v>102</v>
+      </c>
+      <c r="K51" s="5" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="52" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A52">
+        <f t="shared" si="0"/>
+        <v>51</v>
+      </c>
+      <c r="B52" s="6">
+        <v>46318</v>
+      </c>
+      <c r="C52" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="D52" s="4" t="s">
+        <v>112</v>
+      </c>
+      <c r="E52" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="F52" s="4">
+        <v>30</v>
+      </c>
+      <c r="G52" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="H52" s="5" t="s">
+        <v>81</v>
+      </c>
+      <c r="I52">
+        <v>10</v>
+      </c>
+      <c r="J52" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="K52" s="5" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="53" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A53">
+        <f t="shared" si="0"/>
+        <v>52</v>
+      </c>
+      <c r="B53" s="6">
+        <v>46319</v>
+      </c>
+      <c r="C53" s="4" t="s">
+        <v>113</v>
+      </c>
+      <c r="D53" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="E53" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="F53" s="4">
+        <v>20</v>
+      </c>
+      <c r="G53" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="H53" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="I53">
+        <v>9</v>
+      </c>
+      <c r="J53" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="K53" s="5" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="54" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A54">
+        <f t="shared" si="0"/>
+        <v>53</v>
+      </c>
+      <c r="B54" s="6">
+        <v>46319</v>
+      </c>
+      <c r="C54" s="4" t="s">
+        <v>114</v>
+      </c>
+      <c r="D54" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="E54" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="F54" s="4">
+        <v>60</v>
+      </c>
+      <c r="G54" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="H54" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="I54">
+        <v>10</v>
+      </c>
+      <c r="J54" s="5" t="s">
+        <v>102</v>
+      </c>
+      <c r="K54" s="5" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="55" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A55">
+        <f t="shared" si="0"/>
+        <v>54</v>
+      </c>
+      <c r="B55" s="6">
+        <v>46319</v>
+      </c>
+      <c r="C55" s="4" t="s">
+        <v>115</v>
+      </c>
+      <c r="D55" s="4" t="s">
+        <v>82</v>
+      </c>
+      <c r="E55" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="F55" s="4">
+        <v>35</v>
+      </c>
+      <c r="G55" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="H55" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="I55">
+        <v>8</v>
+      </c>
+      <c r="J55" s="5" t="s">
+        <v>89</v>
+      </c>
+      <c r="K55" s="5" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="56" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A56">
+        <f t="shared" si="0"/>
+        <v>55</v>
+      </c>
+      <c r="B56" s="6">
+        <v>46319</v>
+      </c>
+      <c r="C56" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="D56" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="E56" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F56" s="4">
+        <v>45</v>
+      </c>
+      <c r="G56" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="H56" s="5" t="s">
+        <v>81</v>
+      </c>
+      <c r="I56">
+        <v>10</v>
+      </c>
+      <c r="J56" s="5" t="s">
+        <v>102</v>
+      </c>
+      <c r="K56" s="5" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="57" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A57">
+        <f>SUM(A56,1)</f>
+        <v>56</v>
+      </c>
+      <c r="B57" s="6">
+        <v>46320</v>
+      </c>
+      <c r="C57" t="s">
+        <v>21</v>
+      </c>
+      <c r="D57" t="s">
+        <v>72</v>
+      </c>
+      <c r="E57" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="F57" s="8">
+        <v>180</v>
+      </c>
+      <c r="G57" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="H57" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="I57">
+        <v>10</v>
+      </c>
+      <c r="J57" s="5" t="s">
+        <v>89</v>
+      </c>
+      <c r="K57" s="5" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="58" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A58">
+        <f t="shared" ref="A58:A71" si="1">SUM(A57,1)</f>
+        <v>57</v>
+      </c>
+      <c r="B58" s="6">
+        <v>46320</v>
+      </c>
+      <c r="C58" s="9" t="s">
+        <v>105</v>
+      </c>
+      <c r="D58" t="s">
+        <v>110</v>
+      </c>
+      <c r="E58" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="F58" s="8">
+        <v>60</v>
+      </c>
+      <c r="G58" t="s">
+        <v>106</v>
+      </c>
+      <c r="H58" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="I58">
+        <v>7</v>
+      </c>
+      <c r="J58" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="K58" s="5" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="59" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A59">
+        <f t="shared" si="1"/>
+        <v>58</v>
+      </c>
+      <c r="B59" s="6">
+        <v>46320</v>
+      </c>
+      <c r="C59" s="4" t="s">
+        <v>97</v>
+      </c>
+      <c r="D59" s="4" t="s">
+        <v>99</v>
+      </c>
+      <c r="E59" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="F59" s="4">
+        <v>30</v>
+      </c>
+      <c r="G59" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="H59" s="5" t="s">
+        <v>98</v>
+      </c>
+      <c r="I59">
+        <v>9</v>
+      </c>
+      <c r="J59" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="K59" s="5" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="60" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A60">
+        <f t="shared" si="1"/>
+        <v>59</v>
+      </c>
+      <c r="B60" s="6">
+        <v>46320</v>
+      </c>
+      <c r="C60" t="s">
+        <v>33</v>
+      </c>
+      <c r="D60" t="s">
+        <v>117</v>
+      </c>
+      <c r="E60" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F60" s="4">
+        <v>40</v>
+      </c>
+      <c r="G60" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="H60" s="5" t="s">
+        <v>81</v>
+      </c>
+      <c r="I60">
+        <v>10</v>
+      </c>
+      <c r="J60" s="5" t="s">
+        <v>102</v>
+      </c>
+      <c r="K60" s="5" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="61" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A61">
+        <f t="shared" si="1"/>
+        <v>60</v>
+      </c>
+      <c r="B61" s="6">
+        <v>46321</v>
+      </c>
+      <c r="C61" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="D61" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="E61" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F61" s="4">
+        <v>90</v>
+      </c>
+      <c r="G61" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="H61" s="5" t="s">
+        <v>98</v>
+      </c>
+      <c r="I61">
+        <v>9</v>
+      </c>
+      <c r="J61" s="5" t="s">
+        <v>89</v>
+      </c>
+      <c r="K61" s="5" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="62" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A62">
+        <f t="shared" si="1"/>
+        <v>61</v>
+      </c>
+      <c r="B62" s="6">
+        <v>46321</v>
+      </c>
+      <c r="C62" s="9" t="s">
+        <v>35</v>
+      </c>
+      <c r="D62" s="4" t="s">
+        <v>99</v>
+      </c>
+      <c r="E62" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="F62" s="4">
+        <v>50</v>
+      </c>
+      <c r="G62" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="H62" s="5" t="s">
+        <v>98</v>
+      </c>
+      <c r="I62">
+        <v>9</v>
+      </c>
+      <c r="J62" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="K62" s="5" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="63" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A63">
+        <f t="shared" si="1"/>
+        <v>62</v>
+      </c>
+      <c r="B63" s="6">
+        <v>46321</v>
+      </c>
+      <c r="C63" s="9" t="s">
+        <v>79</v>
+      </c>
+      <c r="D63" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="E63" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F63" s="4">
+        <v>20</v>
+      </c>
+      <c r="G63" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="H63" s="5" t="s">
+        <v>98</v>
+      </c>
+      <c r="I63">
+        <v>4</v>
+      </c>
+      <c r="J63" s="5" t="s">
+        <v>89</v>
+      </c>
+      <c r="K63" s="5" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="64" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A64">
+        <f t="shared" si="1"/>
+        <v>63</v>
+      </c>
+      <c r="B64" s="6">
+        <v>46321</v>
+      </c>
+      <c r="C64" t="s">
+        <v>33</v>
+      </c>
+      <c r="D64" t="s">
+        <v>73</v>
+      </c>
+      <c r="E64" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="F64" s="8">
+        <v>45</v>
+      </c>
+      <c r="G64" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="H64" s="5" t="s">
+        <v>81</v>
+      </c>
+      <c r="I64">
+        <v>10</v>
+      </c>
+      <c r="J64" s="5" t="s">
+        <v>102</v>
+      </c>
+      <c r="K64" s="5" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="65" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A65">
+        <f t="shared" si="1"/>
+        <v>64</v>
+      </c>
+      <c r="B65" s="6">
+        <v>46322</v>
+      </c>
+      <c r="C65" t="s">
+        <v>31</v>
+      </c>
+      <c r="D65" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="E65" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F65" s="4">
+        <v>90</v>
+      </c>
+      <c r="G65" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="H65" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="I65">
+        <v>5</v>
+      </c>
+      <c r="J65" s="5" t="s">
+        <v>89</v>
+      </c>
+      <c r="K65" s="5" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="66" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A66">
+        <f t="shared" si="1"/>
+        <v>65</v>
+      </c>
+      <c r="B66" s="6">
+        <v>46322</v>
+      </c>
+      <c r="C66" t="s">
+        <v>104</v>
+      </c>
+      <c r="D66" t="s">
+        <v>109</v>
+      </c>
+      <c r="E66" t="s">
+        <v>41</v>
+      </c>
+      <c r="F66">
+        <v>120</v>
+      </c>
+      <c r="G66" t="s">
+        <v>7</v>
+      </c>
+      <c r="H66" t="s">
+        <v>27</v>
+      </c>
+      <c r="I66">
+        <v>9</v>
+      </c>
+      <c r="J66" t="s">
+        <v>89</v>
+      </c>
+      <c r="K66" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="67" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A67">
+        <f t="shared" si="1"/>
+        <v>66</v>
+      </c>
+      <c r="B67" s="6">
+        <v>46322</v>
+      </c>
+      <c r="C67" t="s">
+        <v>33</v>
+      </c>
+      <c r="D67" t="s">
+        <v>116</v>
+      </c>
+      <c r="E67" t="s">
+        <v>41</v>
+      </c>
+      <c r="F67">
+        <v>30</v>
+      </c>
+      <c r="G67" t="s">
+        <v>11</v>
+      </c>
+      <c r="H67" t="s">
+        <v>81</v>
+      </c>
+      <c r="I67">
+        <v>10</v>
+      </c>
+      <c r="J67" t="s">
+        <v>102</v>
+      </c>
+      <c r="K67" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="68" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A68">
+        <f t="shared" si="1"/>
+        <v>67</v>
+      </c>
+      <c r="B68" s="6">
+        <v>46322</v>
+      </c>
+      <c r="C68" t="s">
+        <v>36</v>
+      </c>
+      <c r="D68" t="s">
+        <v>112</v>
+      </c>
+      <c r="E68" s="9" t="s">
+        <v>8</v>
+      </c>
+      <c r="F68" s="9">
+        <v>20</v>
+      </c>
+      <c r="G68" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="H68" s="9" t="s">
+        <v>81</v>
+      </c>
+      <c r="I68">
+        <v>10</v>
+      </c>
+      <c r="J68" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="K68" s="5" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="69" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A69">
+        <f t="shared" si="1"/>
+        <v>68</v>
+      </c>
+    </row>
+    <row r="70" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A70">
+        <f t="shared" si="1"/>
+        <v>69</v>
+      </c>
+    </row>
+    <row r="71" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A71">
+        <f t="shared" si="1"/>
+        <v>70</v>
       </c>
     </row>
   </sheetData>

</xml_diff>